<commit_message>
chore : minor changes
</commit_message>
<xml_diff>
--- a/VotingConsole/users.xlsx
+++ b/VotingConsole/users.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +449,16 @@
           <t>Vote</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>RegisteredOn</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -471,6 +481,8 @@
           <t>Party A</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -493,6 +505,8 @@
           <t>Party A</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -513,6 +527,84 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>Party B</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>kk</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>kk</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>c27c7ea1-e761-4332-8fde-23d8877b29e7</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Party A</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>555</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>555</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>3ad5e135-7a7f-4ada-9ae2-3ff282a46b1f</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Party A</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>888</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>888</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>dad81b3e-c349-42ad-bffe-da4e3eb9fbd0</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2025-01-25 21:46:52</t>
         </is>
       </c>
     </row>

</xml_diff>